<commit_message>
Admin: amélioration de la gestion des liens et ajout d'upload de documents
- Tableau d'honneur: ajout/suppression de niveaux avec URLs éditables
- Cartes examens: ajout/suppression de cartes avec URLs éditables
- Chers Parents: URL éditable + possibilité d'ajouter des liens supplémentaires
- Infos Pratiques: tous les liens (1er cycle, 2nd cycle, calendrier, footer) avec URLs visibles
- Actualités: liens éditables avec champ URL
- Bouton d'upload de documents (PDF)  à côté de chaque champ URL
- Admin peut maintenant soit entrer une URL manuellement, soit uploader un PDF
</commit_message>
<xml_diff>
--- a/admin-operators-credentials.xlsx
+++ b/admin-operators-credentials.xlsx
@@ -449,13 +449,13 @@
         <v>Oui</v>
       </c>
       <c r="E2" t="str">
-        <v>wyDpU!96jGpCiHeR!H</v>
+        <v>gZSTkPkW</v>
       </c>
       <c r="F2" t="str">
         <v>Oui</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-04-12T15:43:35.113Z</v>
+        <v>2026-04-12T16:21:11.183Z</v>
       </c>
       <c r="H2" t="str">
         <v>/ecqm19-admin</v>
@@ -475,13 +475,13 @@
         <v>Oui</v>
       </c>
       <c r="E3" t="str">
-        <v>ou_fBVWoHa4HpG9QYo</v>
+        <v>VmuHd4VS</v>
       </c>
       <c r="F3" t="str">
         <v>Oui</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-04-12T15:43:35.296Z</v>
+        <v>2026-04-12T16:21:11.320Z</v>
       </c>
       <c r="H3" t="str">
         <v>/ecqm19-admin</v>
@@ -501,13 +501,13 @@
         <v>Oui</v>
       </c>
       <c r="E4" t="str">
-        <v>kVHVVMmaA?AYzP?#FB</v>
+        <v>sPjkwYEK</v>
       </c>
       <c r="F4" t="str">
         <v>Oui</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-04-12T15:43:35.495Z</v>
+        <v>2026-04-12T16:21:11.451Z</v>
       </c>
       <c r="H4" t="str">
         <v>/ecqm19-admin</v>
@@ -527,13 +527,13 @@
         <v>Oui</v>
       </c>
       <c r="E5" t="str">
-        <v>ktkqZh7gZeZU93J7+F</v>
+        <v>uB8N5EMc</v>
       </c>
       <c r="F5" t="str">
         <v>Oui</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-04-12T15:43:35.706Z</v>
+        <v>2026-04-12T16:21:11.582Z</v>
       </c>
       <c r="H5" t="str">
         <v>/ecqm19-admin</v>
@@ -553,13 +553,13 @@
         <v>Oui</v>
       </c>
       <c r="E6" t="str">
-        <v>bEKXsdRNVhZuY=HEz+</v>
+        <v>jqWdXvS6</v>
       </c>
       <c r="F6" t="str">
         <v>Oui</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-04-12T15:43:35.904Z</v>
+        <v>2026-04-12T16:21:11.713Z</v>
       </c>
       <c r="H6" t="str">
         <v>/ecqm19-admin</v>
@@ -579,13 +579,13 @@
         <v>Oui</v>
       </c>
       <c r="E7" t="str">
-        <v>!@7saGeE#CBkKKgNfu</v>
+        <v>cSHYoTE7</v>
       </c>
       <c r="F7" t="str">
         <v>Oui</v>
       </c>
       <c r="G7" t="str">
-        <v>2026-04-12T15:43:36.064Z</v>
+        <v>2026-04-12T16:21:11.855Z</v>
       </c>
       <c r="H7" t="str">
         <v>/ecqm19-admin</v>
@@ -605,13 +605,13 @@
         <v>Oui</v>
       </c>
       <c r="E8" t="str">
-        <v>YspT6n@3KYX+uhxsvB</v>
+        <v>jp2wZN5E</v>
       </c>
       <c r="F8" t="str">
         <v>Oui</v>
       </c>
       <c r="G8" t="str">
-        <v>2026-04-12T15:43:36.229Z</v>
+        <v>2026-04-12T16:21:12.053Z</v>
       </c>
       <c r="H8" t="str">
         <v>/ecqm19-admin</v>
@@ -631,13 +631,13 @@
         <v>Oui</v>
       </c>
       <c r="E9" t="str">
-        <v>y?DMJnWycufihuZeDS</v>
+        <v>YMKUSNsS</v>
       </c>
       <c r="F9" t="str">
         <v>Oui</v>
       </c>
       <c r="G9" t="str">
-        <v>2026-04-12T15:43:36.412Z</v>
+        <v>2026-04-12T16:21:12.218Z</v>
       </c>
       <c r="H9" t="str">
         <v>/ecqm19-admin</v>
@@ -657,13 +657,13 @@
         <v>Oui</v>
       </c>
       <c r="E10" t="str">
-        <v>#bjeia7f3CCXzdq$fh</v>
+        <v>ZgkrEyH4</v>
       </c>
       <c r="F10" t="str">
         <v>Oui</v>
       </c>
       <c r="G10" t="str">
-        <v>2026-04-12T15:43:36.572Z</v>
+        <v>2026-04-12T16:21:12.331Z</v>
       </c>
       <c r="H10" t="str">
         <v>/ecqm19-admin</v>
@@ -683,13 +683,13 @@
         <v>Oui</v>
       </c>
       <c r="E11" t="str">
-        <v>ErRi%GXxY_bjmPngLe</v>
+        <v>gtSb2Wjr</v>
       </c>
       <c r="F11" t="str">
         <v>Oui</v>
       </c>
       <c r="G11" t="str">
-        <v>2026-04-12T15:43:36.725Z</v>
+        <v>2026-04-12T16:21:12.440Z</v>
       </c>
       <c r="H11" t="str">
         <v>/ecqm19-admin</v>

</xml_diff>